<commit_message>
Update Pandas earthquake and meteorite scripts
</commit_message>
<xml_diff>
--- a/filtered_earthquakes_high_risk.xlsx
+++ b/filtered_earthquakes_high_risk.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2115,56 +2115,56 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-03T05:37:23.637Z</t>
+          <t>2026-03-03T12:20:07.033Z</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>27.4027</v>
+        <v>32.14</v>
       </c>
       <c r="C20" t="n">
-        <v>139.8684</v>
+        <v>-101.084</v>
       </c>
       <c r="D20" t="n">
-        <v>500.758</v>
+        <v>8.227499999999999</v>
       </c>
       <c r="E20" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>mb</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>105</v>
+        <v>32</v>
       </c>
       <c r="H20" t="n">
-        <v>134</v>
+        <v>54</v>
       </c>
       <c r="I20" t="n">
-        <v>7.896</v>
+        <v>0.2</v>
       </c>
       <c r="J20" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>us</t>
+          <t>tx</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>us7000s1mj</t>
+          <t>tx2026eixvly</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-03-03T08:05:11.040Z</t>
+          <t>2026-03-05T02:44:00.647Z</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Bonin Islands, Japan region</t>
+          <t>24 km SSW of Westbrook, Texas</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2173,16 +2173,16 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>11.61</v>
+        <v>0.41213581502354</v>
       </c>
       <c r="Q20" t="n">
-        <v>9.101000000000001</v>
+        <v>1.2411064226168</v>
       </c>
       <c r="R20" t="n">
-        <v>0.037</v>
+        <v>0.1</v>
       </c>
       <c r="S20" t="n">
-        <v>201</v>
+        <v>19</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
@@ -2191,98 +2191,362 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>us</t>
+          <t>tx</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>us</t>
+          <t>tx</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>2026-03-03T10:52:23.191Z</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>32.132</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-102.214</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5.9326</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>28</v>
+      </c>
+      <c r="H21" t="n">
+        <v>67</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>tx2026eiuxwb</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-03-04T23:29:24.261Z</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>19 km NW of Midland, Texas</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>earthquake</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>0.62648306355475</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1.3358244551329</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="S21" t="n">
+        <v>13</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-03T08:25:51.770Z</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-98.935</v>
+      </c>
+      <c r="D22" t="n">
+        <v>5.9207</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>25</v>
+      </c>
+      <c r="H22" t="n">
+        <v>70</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>tx2026eiqbql</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-03-03T15:19:04.853Z</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>23 km E of Dilley, Texas</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>earthquake</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>1.8110307766354</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1.0986965460629</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>15</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-03T05:37:23.637Z</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>27.4027</v>
+      </c>
+      <c r="C23" t="n">
+        <v>139.8684</v>
+      </c>
+      <c r="D23" t="n">
+        <v>500.758</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>mb</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>105</v>
+      </c>
+      <c r="H23" t="n">
+        <v>134</v>
+      </c>
+      <c r="I23" t="n">
+        <v>7.896</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>us7000s1mj</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-03-03T08:05:11.040Z</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Bonin Islands, Japan region</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>earthquake</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>9.101000000000001</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="S23" t="n">
+        <v>201</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>2026-03-03T00:11:43.467Z</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B24" t="n">
         <v>25.2893</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C24" t="n">
         <v>124.8906</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D24" t="n">
         <v>10</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E24" t="n">
         <v>5</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>mww</t>
         </is>
       </c>
-      <c r="G21" t="n">
+      <c r="G24" t="n">
         <v>67</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H24" t="n">
         <v>91</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I24" t="n">
         <v>1.084</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J24" t="n">
         <v>0.5</v>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>us</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>us7000s1k2</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>2026-03-03T04:53:04.040Z</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>67 km NW of Hirara, Japan</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>earthquake</t>
         </is>
       </c>
-      <c r="P21" t="n">
+      <c r="P24" t="n">
         <v>5.65</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="Q24" t="n">
         <v>1.773</v>
       </c>
-      <c r="R21" t="n">
+      <c r="R24" t="n">
         <v>0.066</v>
       </c>
-      <c r="S21" t="n">
+      <c r="S24" t="n">
         <v>22</v>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>reviewed</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>us</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>us</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
         <is>
           <t>us</t>
         </is>

</xml_diff>